<commit_message>
Add final test-case result Excel files for Labs 10 & 11
</commit_message>
<xml_diff>
--- a/Langchain-Labs/Lab10(Advanced)/lab10-test-case-results.xlsx
+++ b/Langchain-Labs/Lab10(Advanced)/lab10-test-case-results.xlsx
@@ -31,7 +31,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,13 +61,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -489,7 +497,7 @@
           <t>PASS: First cell verified as pinned pip install</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -516,7 +524,7 @@
           <t>PASS: Code cells verified within 180-line limit</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -543,7 +551,7 @@
           <t>PASS: All companion files verified</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -570,7 +578,7 @@
           <t>PASS: Model factory uses correct endpoint and model</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -597,7 +605,7 @@
           <t>PASS: API key loaded from .env</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -624,7 +632,7 @@
           <t>PASS: UsageCapture initialized empty</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -651,7 +659,7 @@
           <t>PASS: Token recording verified</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -678,7 +686,7 @@
           <t>PASS: get_invoice tool verified</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -705,7 +713,7 @@
           <t>PASS: process_refund tool verified</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -732,7 +740,7 @@
           <t>PASS: check_service_status tool verified</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -759,7 +767,7 @@
           <t>PASS: search_kb tool verified</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -786,7 +794,7 @@
           <t>PASS: get_plan tool verified</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -813,7 +821,7 @@
           <t>PASS: set_seats tool verified</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -840,7 +848,7 @@
           <t>PASS: All six tools verified in ALL_TOOLS</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -867,7 +875,7 @@
           <t>PASS: route_billing tool verified</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -894,7 +902,7 @@
           <t>PASS: route_tech tool verified</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -921,7 +929,7 @@
           <t>PASS: route_account tool verified</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -948,7 +956,7 @@
           <t>PASS: Route-to-node mapping verified</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -975,7 +983,7 @@
           <t>PASS: Supervisor prompt covers all departments</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1002,7 +1010,7 @@
           <t>PASS: Graph compiles with four nodes</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1029,7 +1037,7 @@
           <t>PASS: RoutingState uses add_messages correctly</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1056,7 +1064,7 @@
           <t>PASS: transfer_to_tech returns correct command</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1083,7 +1091,7 @@
           <t>PASS: transfer_to_billing returns correct command</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1110,7 +1118,7 @@
           <t>PASS: Handoff budget guard verified</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1137,7 +1145,7 @@
           <t>PASS: Optional exercise documentation verified</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1164,7 +1172,7 @@
           <t>PASS: Documentation structure complete</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1190,17 +1198,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Gate</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Criterion (AGENTS.md)</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
@@ -1310,12 +1318,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1329,7 +1337,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lab 10: Multi-Agent Coordination</t>
+          <t>Lab 10: Multi-Agent Coordination (Advanced)</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1349,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-14 10:00</t>
+          <t>2026-08-14 11:51</t>
         </is>
       </c>
     </row>

</xml_diff>